<commit_message>
chore: sync user words into Excel and vocab-data
</commit_message>
<xml_diff>
--- a/docs/interview-vocab.xlsx
+++ b/docs/interview-vocab.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24750" windowHeight="10980" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网页原文" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java常用单词" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python常用单词" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FastAPI常用单词" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LangChain常用单词" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python补充" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FastAPI补充" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LangChain与RAG补充" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformer补充" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpenCV补充" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI编程工具补充" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java后端补充" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="全部汇总" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="网页原文" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Java常用单词" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Python常用单词" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="FastAPI常用单词" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="LangChain常用单词" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Python补充" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FastAPI补充" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="LangChain与RAG补充" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Transformer补充" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="OpenCV补充" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="AI编程工具补充" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Java后端补充" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="说明" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1100,7 +1100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J318"/>
+  <dimension ref="A1:J319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17648,6 +17648,58 @@
       <c r="J318" s="2" t="inlineStr">
         <is>
           <t>做登录鉴权和权限控制。</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>一种常见的圆形果实，由Malus domestica树生产，在温和的气候下种植。</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>阿-普-呃-勒</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>/ˈæp.əl/</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>一句话：一种常见的圆形果实，由Malus domestica树生产，在温和的气候下种植。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh Excel community sheet after sync.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/interview-vocab.xlsx
+++ b/docs/interview-vocab.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24750" windowHeight="10980" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="全部汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="网页原文" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Java常用单词" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Python常用单词" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="FastAPI常用单词" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="LangChain常用单词" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Python补充" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="FastAPI补充" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="LangChain与RAG补充" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Transformer补充" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="OpenCV补充" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="AI编程工具补充" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Java后端补充" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="说明" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部汇总" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="社区添加单词" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网页原文" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java常用单词" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python常用单词" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FastAPI常用单词" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LangChain常用单词" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python补充" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FastAPI补充" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LangChain与RAG补充" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformer补充" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpenCV补充" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI编程工具补充" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java后端补充" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -18016,7 +18017,6 @@
           <t>德-诶-勒</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr"/>
       <c r="F326" t="inlineStr">
         <is>
           <t>del</t>
@@ -18049,6 +18049,1956 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>单词</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>用法/解释</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>中文谐音</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>音标</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>发音</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>技术栈</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>重要程度</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>对比词</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>一句话回答</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>检索增强生成：先查资料再生成</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>拉格</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>/ræg/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>微调 / 纯 Prompt</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>用外部知识降低幻觉。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>chunking</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>文本分块，便于嵌入和检索</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>畅-金</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>/ˈtʃʌŋkɪŋ/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>chunk-ing</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>整篇塞上下文</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>把长文档切成可检索片段。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>chunk overlap</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>分块重叠，减少跨段信息丢失</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>畅克-欧-弗-莱普</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>/tʃʌŋk ˈəʊvəlæp/</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>chunk oh-ver-lap</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>无重叠硬切</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>相邻块共享一段边界文本。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>RecursiveCharacterTextSplitter</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>按字符递归切分的常用分块器</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>瑞-克-瑟-西-弗-凯-瑞-克特-斯普利特</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>/rɪˈkɜːsɪv ˈkærəktə tekst ˈsplɪtə/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>ri-kur-siv character text splitter</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>TokenTextSplitter</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>按分隔符优先级递归切块。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>TokenTextSplitter</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>按 token 数切分文本</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>托-肯-泰克斯特-斯普利特</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>/ˈtəʊkən tekst ˈsplɪtə/</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>token text splitter</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>字符切分</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>更贴近模型上下文计量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>embedding model</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>把文本变成向量的模型</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>艾姆-贝-丁-莫-德</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>/ɪmˈbedɪŋ ˈmɒdl/</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>im-bed-ing model</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>生成模型 LLM</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>用于语义检索，不是直接写答案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>vector database</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>向量数据库，存向量并近邻搜索</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>维克特-戴-塔-贝斯</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>/ˈvektə ˈdeɪtəbeɪs/</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>vec-ter day-ta-base</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>关系库 LIKE 查询</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>按相似度找回相关片段。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Facebook 开源向量检索库</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>菲斯</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>/faɪs/</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>fice</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Chroma / Milvus</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>本地快速做向量近邻搜索。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Chroma</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>轻量向量库，开发友好</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>克-罗-玛</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>/ˈkrəʊmə/</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>kro-muh</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>FAISS / pgvector</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>快速搭建本地知识库。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Milvus</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>面向生产的向量数据库</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>米尔-弗斯</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>/ˈmɪlvəs/</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>mil-vus</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>大规模向量检索可选用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>pgvector</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PostgreSQL 向量扩展</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>皮-吉-维克特</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>/ˌpiː dʒiː ˈvektə/</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>P-G vector</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>专用向量库</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>业务库和向量库一体。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>similarity search</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>相似度搜索</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>西-米-拉-瑞-提-瑟奇</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>/ˌsɪməˈlærəti sɜːtʃ/</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>sim-i-la-ri-tee search</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>关键词搜索</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>按向量距离找最相近文档。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>hybrid search</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>混合检索：关键词+向量</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>海-布瑞德-瑟奇</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>/ˈhaɪbrɪd sɜːtʃ/</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>hi-brid search</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>纯向量检索</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>专名靠词，语义靠向量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>经典关键词相关性算法</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>比-艾姆-吐-五</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>/ˌbiː em twenti ˈfaɪv/</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>B-M twenty-five</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF / 向量检索</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>稀疏检索常用打分函数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>rerank</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>对召回结果重排序</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>瑞-兰克</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>/ˌriːˈræŋk/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>ree-rank</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>只靠向量 Top-K</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>用更准模型精排候选片段。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Top-K</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>取相似度最高的 K 条</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>托普-凯</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>/tɒp keɪ/</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>top kay</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>阈值过滤</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>控制送进 Prompt 的片段数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>metadata filtering</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>按元数据过滤检索结果</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>梅-塔-戴-塔-菲-欧-特-林</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>/ˈmetədeɪtə ˈfɪltərɪŋ/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>meta-data filtering</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>纯相似度</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>按来源/时间/类目缩小范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>citation</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>答案引用检索来源</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>赛-泰-申</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>/saɪˈteɪʃən/</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>sigh-tay-shun</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>无引用生成</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>可追溯，降低瞎编。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>hallucination</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>幻觉：编造不实内容</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>哈-卢-西-内-申</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>/həˌluːsɪˈneɪʃən/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>huh-loo-si-nay-shun</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>拒答 / 检索约束</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>RAG 和人审就是为压它。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>LCEL</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>LangChain 表达式语言，管道组合组件</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>艾欧西伊艾欧</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>/ˌel siː iː ˈel/</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>L-C-E-L</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>老版 Chain 类</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>用 | 把 prompt、模型、解析串起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>PromptTemplate</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>提示词模板</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>普-罗姆普特-坦普雷特</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>/prɒmpt ˈtemplət/</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>prompt tem-plit</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>硬编码字符串</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>把变量填进固定提示结构。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>ChatPromptTemplate</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>多角色聊天提示模板</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>恰特-普-罗姆普特-坦普雷特</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>/tʃæt prɒmpt ˈtemplət/</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>chat prompt tem-plit</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>PromptTemplate</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>组装 system/user/assistant 消息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>OutputParser</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>把模型输出解析成结构化数据</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>奥特-普特-帕-瑟</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>/ˈaʊtpʊt ˈpɑːsə/</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>out-put par-ser</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>手工正则抠文本</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>稳定提取 JSON/对象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>tool calling</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>工具调用，模型决定调哪个函数</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>图-欧-考-林</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>/tuːl ˈkɔːlɪŋ/</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>tool call-ing</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>纯文本回答</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>让模型联动检索、计算、API。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>对话记忆，保存历史上下文</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>梅-莫-瑞</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>/ˈmeməri/</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>mem-uh-ree</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>无状态单轮</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>支持多轮连续对话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>StateGraph</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>状态图，LangGraph 编排核心</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>斯忒特-格-拉夫</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>/steɪt ɡrɑːf/</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>state graph</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>线性 Chain</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>用节点和边描述复杂流程。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>checkpoint</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>检查点，持久化图状态</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>切克-波因特</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>/ˈtʃekpɔɪnt/</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>check-point</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>无状态重跑</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>支持暂停恢复和排错回放。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>interrupt</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>中断，人在回路时挂起</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>因-特-拉普特</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>/ˌɪntəˈrʌpt/</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>in-tuh-rupt</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>全自动执行</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>关键步骤等人审再继续。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>human-in-the-loop</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>人在回路，人工确认关键步骤</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>休-曼-因-泽-鲁普</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>/ˈhjuːmən ɪn ðə luːp/</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>human in the loop</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>全自动 Agent</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>高风险操作必须人审。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>conditional edge</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>条件边，按状态路由下一节点</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>康-迪-申-纳-欧-艾奇</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>/kənˈdɪʃənl edʒ/</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>kun-dish-uh-nul edge</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>固定顺序边</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>实现分支和重试。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>本地运行开源大模型的工具</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>欧-拉-玛</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>/əˈlɑːmə/</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>uh-lah-muh</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>云端 API</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>本机一键 pull/run 模型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI API</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI 兼容的大模型接口</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>欧-潘-诶-诶皮艾</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>/ˈəʊpən eɪ aɪ ˈeɪ piː aɪ/</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>open AI A-P-I</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>本地推理</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>用 HTTP 调云端对话/嵌入模型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>温度，控制输出随机性</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>坦-普-拉-切</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>/ˈtemprətʃə/</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>tem-pruh-chur</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>top_p</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>越高越发散，越低越稳。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>top_p</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>核采样，按概率质量截断</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>托普-皮</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>/tɒp piː/</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>top pee</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>另一种控制多样性的参数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>max_tokens</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>最大生成 token 数</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>麦克斯-托-肯斯</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>/mæks ˈtəʊkənz/</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>max tokens</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>常问</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>上下文窗口</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>限制回答长度和费用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>模型</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>流式输出，边生成边返回</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>斯-特-瑞-明</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>/ˈstriːmɪŋ/</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>stream-ing</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>一次性返回</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>降低首字等待，体验更好。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19426,7 +21376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20388,7 +22338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21038,7 +22988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23144,7 +25094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23463,6 +25413,468 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>单词</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>用法/解释</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>中文谐音</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>音标</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>发音</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>技术栈</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>重要程度</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>对比词</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>一句话回答</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>添加的行为或实例。</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>阿-德</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>/æd/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>coalesce / join / unite</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>一句话：添加的行为或实例。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>一种常见的圆形果实，由Malus domestica树生产，在温和的气候下种植。</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>阿-普-呃-勒</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>/ˈæp.əl/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>一句话：一种常见的圆形果实，由Malus domestica树生产，在温和的气候下种植。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>（有时大写）非洲人、原住民或毛利人后裔；皮肤黝黑的人。</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>布-勒-克</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>/blak/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>blackball / blacklist / blacken</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>一句话：（有时大写）非洲人、原住民或毛利人后裔；皮肤黝黑的人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>del</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>del：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>德-诶-勒</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>del</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>一句话：del：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>delete</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>delete：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>德-诶-勒-诶-特-诶</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>delete</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>一句话：delete：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>idemmode</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>idemmode：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>伊-德-诶-姆-姆-德-诶</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>idemmode</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>一句话：idemmode：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IS：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>伊-斯</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>一句话：IS：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>社区投稿</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pink：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>普-伊-恩-克</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>一句话：pink：技术面试常见术语，建议结合项目场景理解。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27388,7 +29800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29442,7 +31854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31340,7 +33752,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -33030,7 +35442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35708,7 +38120,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36722,7 +39134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37838,1954 +40250,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>单词</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>用法/解释</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>中文谐音</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>音标</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>发音</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>技术栈</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>重要程度</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>对比词</t>
-        </is>
-      </c>
-      <c r="J1" s="6" t="inlineStr">
-        <is>
-          <t>一句话回答</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>检索增强生成：先查资料再生成</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>拉格</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>/ræg/</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>rag</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>微调 / 纯 Prompt</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>用外部知识降低幻觉。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>chunking</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>文本分块，便于嵌入和检索</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>畅-金</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>/ˈtʃʌŋkɪŋ/</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>chunk-ing</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>整篇塞上下文</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>把长文档切成可检索片段。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>chunk overlap</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>分块重叠，减少跨段信息丢失</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>畅克-欧-弗-莱普</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>/tʃʌŋk ˈəʊvəlæp/</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>chunk oh-ver-lap</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>无重叠硬切</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>相邻块共享一段边界文本。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>RecursiveCharacterTextSplitter</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>按字符递归切分的常用分块器</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>瑞-克-瑟-西-弗-凯-瑞-克特-斯普利特</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>/rɪˈkɜːsɪv ˈkærəktə tekst ˈsplɪtə/</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>ri-kur-siv character text splitter</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>TokenTextSplitter</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>按分隔符优先级递归切块。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>TokenTextSplitter</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>按 token 数切分文本</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>托-肯-泰克斯特-斯普利特</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>/ˈtəʊkən tekst ˈsplɪtə/</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>token text splitter</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>字符切分</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>更贴近模型上下文计量。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>embedding model</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>把文本变成向量的模型</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>艾姆-贝-丁-莫-德</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>/ɪmˈbedɪŋ ˈmɒdl/</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>im-bed-ing model</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>生成模型 LLM</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>用于语义检索，不是直接写答案。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>vector database</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>向量数据库，存向量并近邻搜索</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>维克特-戴-塔-贝斯</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>/ˈvektə ˈdeɪtəbeɪs/</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>vec-ter day-ta-base</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>关系库 LIKE 查询</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>按相似度找回相关片段。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>FAISS</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Facebook 开源向量检索库</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>菲斯</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>/faɪs/</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>fice</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Chroma / Milvus</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>本地快速做向量近邻搜索。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Chroma</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>轻量向量库，开发友好</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>克-罗-玛</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>/ˈkrəʊmə/</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>kro-muh</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>FAISS / pgvector</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>快速搭建本地知识库。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Milvus</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>面向生产的向量数据库</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>米尔-弗斯</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>/ˈmɪlvəs/</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>mil-vus</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>了解</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>FAISS</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>大规模向量检索可选用。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>pgvector</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>PostgreSQL 向量扩展</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>皮-吉-维克特</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>/ˌpiː dʒiː ˈvektə/</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>P-G vector</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>专用向量库</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>业务库和向量库一体。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>similarity search</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>相似度搜索</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>西-米-拉-瑞-提-瑟奇</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>/ˌsɪməˈlærəti sɜːtʃ/</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>sim-i-la-ri-tee search</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>关键词搜索</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>按向量距离找最相近文档。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>hybrid search</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>混合检索：关键词+向量</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>海-布瑞德-瑟奇</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>/ˈhaɪbrɪd sɜːtʃ/</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>hi-brid search</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>纯向量检索</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>专名靠词，语义靠向量。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>BM25</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>经典关键词相关性算法</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>比-艾姆-吐-五</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>/ˌbiː em twenti ˈfaɪv/</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>B-M twenty-five</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>TF-IDF / 向量检索</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>稀疏检索常用打分函数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>rerank</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>对召回结果重排序</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>瑞-兰克</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>/ˌriːˈræŋk/</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>ree-rank</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>只靠向量 Top-K</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>用更准模型精排候选片段。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Top-K</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>取相似度最高的 K 条</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>托普-凯</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>/tɒp keɪ/</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>top kay</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>阈值过滤</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>控制送进 Prompt 的片段数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>metadata filtering</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>按元数据过滤检索结果</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>梅-塔-戴-塔-菲-欧-特-林</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>/ˈmetədeɪtə ˈfɪltərɪŋ/</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>meta-data filtering</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>纯相似度</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>按来源/时间/类目缩小范围。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>答案引用检索来源</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>赛-泰-申</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>/saɪˈteɪʃən/</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>sigh-tay-shun</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>无引用生成</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>可追溯，降低瞎编。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>RAG</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>hallucination</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>幻觉：编造不实内容</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>哈-卢-西-内-申</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>/həˌluːsɪˈneɪʃən/</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>huh-loo-si-nay-shun</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>拒答 / 检索约束</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>RAG 和人审就是为压它。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>LCEL</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>LangChain 表达式语言，管道组合组件</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>艾欧西伊艾欧</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>/ˌel siː iː ˈel/</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>L-C-E-L</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>老版 Chain 类</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>用 | 把 prompt、模型、解析串起来。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>PromptTemplate</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>提示词模板</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>普-罗姆普特-坦普雷特</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>/prɒmpt ˈtemplət/</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>prompt tem-plit</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>硬编码字符串</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>把变量填进固定提示结构。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>ChatPromptTemplate</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>多角色聊天提示模板</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>恰特-普-罗姆普特-坦普雷特</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>/tʃæt prɒmpt ˈtemplət/</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>chat prompt tem-plit</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>PromptTemplate</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>组装 system/user/assistant 消息。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>OutputParser</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>把模型输出解析成结构化数据</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>奥特-普特-帕-瑟</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>/ˈaʊtpʊt ˈpɑːsə/</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>out-put par-ser</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>手工正则抠文本</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>稳定提取 JSON/对象。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>tool calling</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>工具调用，模型决定调哪个函数</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>图-欧-考-林</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>/tuːl ˈkɔːlɪŋ/</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>tool call-ing</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>纯文本回答</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>让模型联动检索、计算、API。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>对话记忆，保存历史上下文</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>梅-莫-瑞</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>/ˈmeməri/</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>mem-uh-ree</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>无状态单轮</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>支持多轮连续对话。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>LangGraph</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>StateGraph</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>状态图，LangGraph 编排核心</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>斯忒特-格-拉夫</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>/steɪt ɡrɑːf/</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>state graph</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>线性 Chain</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>用节点和边描述复杂流程。</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>LangGraph</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>checkpoint</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>检查点，持久化图状态</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>切克-波因特</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>/ˈtʃekpɔɪnt/</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>check-point</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>无状态重跑</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>支持暂停恢复和排错回放。</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>LangGraph</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>interrupt</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>中断，人在回路时挂起</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>因-特-拉普特</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>/ˌɪntəˈrʌpt/</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>in-tuh-rupt</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>全自动执行</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>关键步骤等人审再继续。</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>LangGraph</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>human-in-the-loop</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>人在回路，人工确认关键步骤</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>休-曼-因-泽-鲁普</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>/ˈhjuːmən ɪn ðə luːp/</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>human in the loop</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>全自动 Agent</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>高风险操作必须人审。</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>LangGraph</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>conditional edge</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>条件边，按状态路由下一节点</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>康-迪-申-纳-欧-艾奇</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>/kənˈdɪʃənl edʒ/</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>kun-dish-uh-nul edge</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>固定顺序边</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>实现分支和重试。</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>模型</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Ollama</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>本地运行开源大模型的工具</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>欧-拉-玛</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>/əˈlɑːmə/</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>uh-lah-muh</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>云端 API</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>本机一键 pull/run 模型。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>模型</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>OpenAI API</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>OpenAI 兼容的大模型接口</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>欧-潘-诶-诶皮艾</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>/ˈəʊpən eɪ aɪ ˈeɪ piː aɪ/</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>open AI A-P-I</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>本地推理</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>用 HTTP 调云端对话/嵌入模型。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>模型</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>温度，控制输出随机性</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>坦-普-拉-切</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>/ˈtemprətʃə/</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>tem-pruh-chur</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>top_p</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>越高越发散，越低越稳。</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>模型</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>top_p</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>核采样，按概率质量截断</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>托普-皮</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>/tɒp piː/</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>top pee</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>了解</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>另一种控制多样性的参数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>模型</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>max_tokens</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>最大生成 token 数</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>麦克斯-托-肯斯</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>/mæks ˈtəʊkənz/</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>max tokens</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>常问</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>上下文窗口</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>限制回答长度和费用。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>模型</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>streaming</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>流式输出，边生成边返回</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>斯-特-瑞-明</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>/ˈstriːmɪŋ/</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>stream-ing</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>必问</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>一次性返回</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>降低首字等待，体验更好。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Ensure site-added words sync into Excel community sheet.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/interview-vocab.xlsx
+++ b/docs/interview-vocab.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24750" windowHeight="10980" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="全部汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="社区添加单词" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="网页原文" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Java常用单词" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Python常用单词" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FastAPI常用单词" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="LangChain常用单词" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Python补充" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FastAPI补充" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="LangChain与RAG补充" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Transformer补充" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="OpenCV补充" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AI编程工具补充" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Java后端补充" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="说明" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部汇总" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="社区添加单词" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网页原文" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java常用单词" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python常用单词" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FastAPI常用单词" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LangChain常用单词" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python补充" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FastAPI补充" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LangChain与RAG补充" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transformer补充" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpenCV补充" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI编程工具补充" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java后端补充" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -18205,7 +18205,6 @@
           <t>斯-特-尔-乌-格-格-勒-诶</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr"/>
       <c r="F330" t="inlineStr">
         <is>
           <t>struggle</t>

</xml_diff>